<commit_message>
update tampilan dashboard, demografi, template import gaji, pengaturan, default penamaan choose file slip gaji
</commit_message>
<xml_diff>
--- a/public/assets/template-import-gaji.xlsx
+++ b/public/assets/template-import-gaji.xlsx
@@ -497,17 +497,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Tambahan 1</t>
+          <t>Tunjangan Jabatan</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Tambahan 2</t>
+          <t>Tunjangan Bansos</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Tambahan 3</t>
+          <t>Tunjangan Managerial</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -597,87 +597,87 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 1</t>
+          <t>BP JAMSOSTEK (JHT: 2%); (JP: 1%)</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 2</t>
+          <t>BPJS-Kshtn (JK:1%)</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 3</t>
+          <t>BNI (DPLK Simponi)</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 4</t>
+          <t>KSU Kel. Mitratani</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 5</t>
+          <t>Iuran Anggota SPA</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 6</t>
+          <t>BTN (KPR)</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 7</t>
+          <t>BRI Cab Jember (Briguna)</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 8</t>
+          <t>BRI Unit Serut (Golbertap)</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 9</t>
+          <t>Bank BSM (Pembiayaan Syariah)</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 10</t>
+          <t>Pengembalian Gaji (Kary Renbang)</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 11</t>
+          <t>Iuran IIKB</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 12</t>
+          <t>Potongan Kopkar PTPN I R5</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 13</t>
+          <t>Pengembalian Bonus Thn 2023</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 14</t>
+          <t>Potongan Dapenbun</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 15</t>
+          <t>Potongan gaji (Masjid)</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 16</t>
+          <t>Potongan Waring</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>Potongan 17</t>
+          <t>Pembelian Pengembalian DPU</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
@@ -3715,22 +3715,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Tambahan</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Potongan</t>
         </is>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Tambahan 1</t>
+          <t>Tunjangan Jabatan</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Potongan 1</t>
+          <t>BP JAMSOSTEK (JHT: 2%); (JP: 1%)</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Tambahan 2</t>
+          <t>Tunjangan Bansos</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Potongan 2</t>
+          <t>BPJS-Kshtn (JK:1%)</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3778,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Tambahan 3</t>
+          <t>Tunjangan Managerial</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Potongan 3</t>
+          <t>BNI (DPLK Simponi)</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3804,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Potongan 4</t>
+          <t>KSU Kel. Mitratani</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Potongan 5</t>
+          <t>Iuran Anggota SPA</t>
         </is>
       </c>
     </row>
@@ -3840,7 +3840,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Potongan 6</t>
+          <t>BTN (KPR)</t>
         </is>
       </c>
     </row>
@@ -3858,7 +3858,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Potongan 7</t>
+          <t>BRI Cab Jember (Briguna)</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3876,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Potongan 8</t>
+          <t>BRI Unit Serut (Golbertap)</t>
         </is>
       </c>
     </row>
@@ -3894,7 +3894,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Potongan 9</t>
+          <t>Bank BSM (Pembiayaan Syariah)</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3912,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Potongan 10</t>
+          <t>Pengembalian Gaji (Kary Renbang)</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3930,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Potongan 11</t>
+          <t>Iuran IIKB</t>
         </is>
       </c>
     </row>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Potongan 12</t>
+          <t>Potongan Kopkar PTPN I R5</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Potongan 13</t>
+          <t>Pengembalian Bonus Thn 2023</t>
         </is>
       </c>
     </row>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Potongan 14</t>
+          <t>Potongan Dapenbun</t>
         </is>
       </c>
     </row>
@@ -4002,7 +4002,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Potongan 15</t>
+          <t>Potongan gaji (Masjid)</t>
         </is>
       </c>
     </row>
@@ -4020,7 +4020,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Potongan 16</t>
+          <t>Potongan Waring</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4038,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Potongan 17</t>
+          <t>Pembelian Pengembalian DPU</t>
         </is>
       </c>
     </row>

</xml_diff>